<commit_message>
web: width/alignment write-back script and fill-in sheet with alignment columns
</commit_message>
<xml_diff>
--- a/web/docs/sheet-column-widths.xlsx
+++ b/web/docs/sheet-column-widths.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -432,6 +432,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,6 +467,16 @@
           <t>新宽度（像素）</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>当前对齐方式</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>新对齐方式</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -488,9 +500,15 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>居左</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -514,9 +532,15 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>居左</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -540,9 +564,15 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>居左</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -566,9 +596,15 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>居左</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -592,9 +628,15 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>居右</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -618,9 +660,15 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>居左</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -644,9 +692,15 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -670,9 +724,15 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -696,9 +756,15 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -722,9 +788,15 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -748,9 +820,15 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -774,9 +852,15 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -800,9 +884,15 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -826,9 +916,15 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -852,9 +948,15 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -878,9 +980,15 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -904,9 +1012,15 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -930,9 +1044,15 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -956,9 +1076,15 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -982,9 +1108,15 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1008,9 +1140,15 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>主水居右、客水居左</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1034,9 +1172,15 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1060,9 +1204,15 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>大球居右、小球居左</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1086,9 +1236,15 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1112,9 +1268,15 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>胜居右、平居中、负居左</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1138,9 +1300,15 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1164,9 +1332,15 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1190,9 +1364,15 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>胜居右、平居中、负居左</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1216,9 +1396,15 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>居中</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1242,9 +1428,15 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>胜居右、平居中、负居左</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>